<commit_message>
Add testcase and automation code
</commit_message>
<xml_diff>
--- a/testcase/Trello_TestCase_CreateANewList_v1.0.xlsx
+++ b/testcase/Trello_TestCase_CreateANewList_v1.0.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\01AutomationTest\03Practices\03Git\TrelloApiAutomation\testcase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4830480E-2CCB-47E2-AABC-D622ADD57997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA55869-91CD-48C5-BC4E-9702A2F00899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="868" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestCase-CreateBoard" sheetId="1" r:id="rId1"/>
-    <sheet name="TestCase-CreateList" sheetId="6" r:id="rId2"/>
-    <sheet name="Trello API-Field Validation" sheetId="2" r:id="rId3"/>
+    <sheet name="TestCase-CreateList" sheetId="1" r:id="rId1"/>
+    <sheet name="CreateList-FieldValidation" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="145621"/>
   <extLst>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
   <si>
     <t>TCID</t>
   </si>
@@ -126,37 +125,6 @@
   </si>
   <si>
     <t>Error message</t>
-  </si>
-  <si>
-    <t>2. Status code and message are displayed correctly:
-- Status Code = 405 (Invalid Method)
-- Message = "No route found for \"POST http://dog.ceo/api/breeds/list/all\": Method Not Allowed (Allow: GET, HEAD) with code: 0"</t>
-  </si>
-  <si>
-    <t>2. Status code and message are displayed correctly:
-- Status Code = 404
-- Message = "No route found for \"GET http://dog.ceo/api/breeds/list/all/check\" with code: 0"</t>
-  </si>
-  <si>
-    <t>Create a new board</t>
-  </si>
-  <si>
-    <t>1. Send request with:
-- valid URL= https://api.trello.com/1/boards?token=ATTAb420992e7d1af6eca93258596c690c760cc1b6bbd75b8d1a8f1af82f3b7eccf207E67C6A&amp;key=f5669804350a0d79b456664598fa3b90
-- invalid Method = GET
-2. Check Status code and message in response.</t>
-  </si>
-  <si>
-    <t>1. Send request with:
-- valid URL =https://api.trello.com/1/boards?token=ATTAb420992e7d1af6eca93258596c690c760cc1b6bbd75b8d1a8f1af82f3b7eccf207E67C6A&amp;key=f5669804350a0d79b456664598fa3b90
-- valid Method = POST
-2. Check response.</t>
-  </si>
-  <si>
-    <t>1. Send request with:
-- invalid URL= https://api.trello.com/1/board
-- valid Method = POST
-2. Check Status code and message in response.</t>
   </si>
   <si>
     <t>2. Response body is returned correctly.
@@ -166,100 +134,88 @@
 Refer file: CreateANewBoardResponseBody.json</t>
   </si>
   <si>
-    <t>"Bài tập về nhà"</t>
-  </si>
-  <si>
     <t xml:space="preserve"> invalid value for name</t>
   </si>
   <si>
     <t>Nhập sai - Thiếu field(test cho case name là require)</t>
   </si>
   <si>
-    <t>defaultList</t>
-  </si>
-  <si>
-    <t>"true"</t>
-  </si>
-  <si>
     <t>Không nhập field - API mặc định là true</t>
   </si>
   <si>
     <t>Nhập null - API vẫn mặc định là true</t>
   </si>
   <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>Nhập đúng - Không có defaultList</t>
-  </si>
-  <si>
     <t>API mặc định là true</t>
   </si>
   <si>
+    <t xml:space="preserve">token =your token
+key = your key </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Status code and message are displayed correctly:
+- Status Code = 403 (Invalid Method)
+- Message = </t>
+  </si>
+  <si>
+    <t>2. Status code and message are displayed correctly:
+- Status Code = 401 Unauthorized
+- Message = "missing scopes"</t>
+  </si>
+  <si>
+    <t>token</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>key</t>
+  </si>
+  <si>
+    <t>Invalid app token</t>
+  </si>
+  <si>
+    <t>invalid key</t>
+  </si>
+  <si>
+    <t>missing scopes</t>
+  </si>
+  <si>
     <t>"Bài chưa làm"</t>
   </si>
   <si>
-    <t>idBoard</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> invalid value for idBoard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nhập sai kiểu dữ liệu </t>
-  </si>
-  <si>
-    <t>Field Validation - Create a new board</t>
-  </si>
-  <si>
-    <t>Field Validation - Create a new list</t>
+    <t>1. Send request with:
+- valid URL =https://api.trello.com/1/lists?token=ATTAaef390986ed8a0c2d34541293e8423005138d3e26802b165932796f6f240a5513CDC7D24&amp;key=f6832e3c462c191601e53abfe5849652
+- valid Method = POST
+2. Check response.</t>
   </si>
   <si>
     <t>Create a new list</t>
   </si>
   <si>
     <t>1. Send request with:
-- valid URL= https://trello.com/1/lists?token=ATTAb420992e7d1af6eca93258596c690c760cc1b6bbd75b8d1a8f1af82f3b7eccf207E67C6A&amp;key=f5669804350a0d79b456664598fa3b90
+- valid URL= https://api.trello.com/1/lists?token=&lt;token&gt;&amp;key=&lt;key&gt;
 - invalid Method = GET
 2. Check Status code and message in response.</t>
   </si>
   <si>
-    <t>2. Status code and message are displayed correctly:
-- Status Code = 401
-- Message = "missing scopes"</t>
-  </si>
-  <si>
     <t>1. Send request with:
-- valid URL =https://trello.com/1/lists?token=ATTAb420992e7d1af6eca93258596c690c760cc1b6bbd75b8d1a8f1af82f3b7eccf207E67C6A&amp;key=f5669804350a0d79b456664598fa3b90
-- valid Method = POST
-2. Check response.</t>
-  </si>
-  <si>
-    <t>1. Send request with:
-- Valid URL = https://trello.com/1/lists?token=ATTAb420992e7d1af6eca93258596c690c760cc1b6bbd75b8d1a8f1af82f3b7eccf207E67C6A&amp;key=f5669804350a0d79b456664598fa3b90
-- Valid Method = POST
-- Data as [Trello API-Field Validation] sheet
-2. Check Status code and message in response.</t>
-  </si>
-  <si>
-    <t>2. Status code and message are displayed correctly. ( [Trello API-Field Validation] sheet)</t>
-  </si>
-  <si>
-    <t>2. Status code and message are displayed correctly:
-- Status Code = 403 (Invalid Method)
-- Message = "The request could not be satisfied"</t>
-  </si>
-  <si>
-    <t>1. Send request with:
-- invalid URL= https://trello.com/1/board
+- invalid URL= https://api.trello.com/1/list
 - valid Method = POST
 2. Check Status code and message in response.</t>
+  </si>
+  <si>
+    <t>Field Validation - Create a new list</t>
+  </si>
+  <si>
+    <t>idBoard</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,6 +265,12 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -330,7 +292,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -388,12 +350,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -409,7 +382,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -423,20 +395,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -660,7 +627,7 @@
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="18.54296875" customWidth="1"/>
     <col min="3" max="3" width="24.81640625" customWidth="1"/>
-    <col min="4" max="4" width="43.08984375" customWidth="1"/>
+    <col min="4" max="4" width="57.7265625" customWidth="1"/>
     <col min="5" max="5" width="47.81640625" customWidth="1"/>
     <col min="6" max="6" width="19.08984375" customWidth="1"/>
     <col min="7" max="7" width="28.453125" customWidth="1"/>
@@ -702,18 +669,20 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="3"/>
+        <v>50</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="G2" s="3"/>
       <c r="H2" s="5" t="s">
         <v>10</v>
@@ -748,10 +717,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -784,14 +753,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>38</v>
+      <c r="D4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -1860,155 +1829,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6648DE38-4C6F-4D3B-A630-6C5DA9D37061}">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="4.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="14.90625" customWidth="1"/>
-    <col min="4" max="4" width="41.6328125" customWidth="1"/>
-    <col min="5" max="5" width="42.81640625" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" customWidth="1"/>
-    <col min="7" max="7" width="17.90625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="123.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="72" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="134" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H5" xr:uid="{98CD6D15-B454-4C71-8A09-DCF52530C6CF}">
-      <formula1>"High,Medium,Low"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G999"/>
+  <dimension ref="A1:G985"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.81640625" customWidth="1"/>
@@ -2023,7 +1845,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -2033,458 +1855,278 @@
       <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="11">
+      <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="11">
+      <c r="C3" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="10">
         <v>200</v>
       </c>
-      <c r="E3" s="13"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11" t="s">
+      <c r="E3" s="12"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11">
+      <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="10">
         <v>400</v>
       </c>
-      <c r="E4" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11" t="s">
-        <v>41</v>
+      <c r="E4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11">
+      <c r="A5" s="10">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="10">
         <v>400</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="E5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
     </row>
     <row r="6" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>4</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="10">
         <v>400</v>
       </c>
-      <c r="E6" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="14"/>
+      <c r="E6" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="10">
         <v>400</v>
       </c>
-      <c r="E7" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="12"/>
+      <c r="E7" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11"/>
     </row>
     <row r="8" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11">
-        <v>6</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="11">
-        <v>200</v>
-      </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="14" t="s">
-        <v>30</v>
+      <c r="A8" s="10">
+        <v>9</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="10">
+        <v>400</v>
+      </c>
+      <c r="E8" s="14"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="11" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11">
-        <v>7</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="D9" s="11">
-        <v>200</v>
-      </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="14"/>
+      <c r="A9" s="10">
+        <v>10</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="10">
+        <v>400</v>
+      </c>
+      <c r="E9" s="14"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="13" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11">
-        <v>8</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="11">
-        <v>200</v>
-      </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="14" t="s">
-        <v>47</v>
+      <c r="A10" s="10">
+        <v>11</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="10">
+        <v>400</v>
+      </c>
+      <c r="E10" s="14"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="11">
-        <v>9</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="16" t="s">
+      <c r="A11" s="10">
+        <v>12</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="11">
-        <v>200</v>
-      </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="12" t="s">
-        <v>44</v>
-      </c>
+      <c r="D11" s="10">
+        <v>401</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="10"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="11">
-        <v>10</v>
-      </c>
-      <c r="B12" s="12" t="s">
+      <c r="A12" s="10">
+        <v>13</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="11">
-        <v>200</v>
-      </c>
-      <c r="E12" s="15"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="14" t="s">
-        <v>45</v>
-      </c>
+      <c r="D12" s="10">
+        <v>401</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="11">
-        <v>11</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="11">
-        <v>200</v>
-      </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="12" t="s">
-        <v>48</v>
-      </c>
+      <c r="A13" s="10">
+        <v>14</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="10">
+        <v>401</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="10"/>
+      <c r="G13" s="11"/>
     </row>
     <row r="14" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G14" s="7"/>
+      <c r="A14" s="10">
+        <v>15</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="10">
+        <v>401</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="10"/>
+      <c r="G14" s="11"/>
     </row>
     <row r="15" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G15" s="7"/>
+      <c r="D15" s="16"/>
     </row>
-    <row r="16" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-    </row>
-    <row r="17" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="11">
-        <v>1</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="11">
-        <v>200</v>
-      </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="11">
-        <v>2</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="11">
-        <v>400</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="11">
-        <v>3</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="11">
-        <v>400</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-    </row>
-    <row r="21" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="11">
-        <v>4</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="11">
-        <v>400</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="14"/>
-    </row>
-    <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="11">
-        <v>5</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="11">
-        <v>400</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12"/>
-    </row>
-    <row r="23" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="11">
-        <v>6</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="11">
-        <v>400</v>
-      </c>
-      <c r="E23" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="14"/>
-    </row>
-    <row r="24" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="11">
-        <v>7</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="11">
-        <v>400</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F24" s="11"/>
-      <c r="G24" s="14"/>
-    </row>
-    <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="11">
-        <v>8</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="11">
-        <v>400</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="11"/>
-      <c r="G25" s="14"/>
-    </row>
-    <row r="26" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="11">
-        <v>9</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="11">
-        <v>400</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F26" s="11"/>
-      <c r="G26" s="12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="29" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="31" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="32" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="20" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="21" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="22" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="23" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="26" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="27" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="28" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="29" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -3438,33 +3080,17 @@
     <row r="983" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="984" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="985" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="986" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="987" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="988" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="989" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="990" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="991" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="992" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="993" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A16:G16"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F13 F18:F26" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F14" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"PASSED,FAILED"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="eve.holt@reqres.in" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="C18" r:id="rId2" display="eve.holt@reqres.in" xr:uid="{93670E6E-B0A1-4C6E-ADAA-7B3426A83115}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>